<commit_message>
Backup: Versi 1.9.26+49 - Standarisasi RT/RW 3 digit, sorting detail dashboard, dan validasi duplikasi Kepala Keluarga/KRT
</commit_message>
<xml_diff>
--- a/data/daftar ketua RT RW.xlsx
+++ b/data/daftar ketua RT RW.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Project\DAWIS\data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{788915F4-8843-476D-B55E-B9D2C12D760F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD30BBB-5FD8-4D54-B59D-6D302A46D1A4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{65BC4B0E-25BE-4BCF-93A8-537B14F26BBC}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="244" uniqueCount="187">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="246" uniqueCount="189">
   <si>
     <t>RW</t>
   </si>
@@ -600,19 +600,32 @@
   </si>
   <si>
     <t>539.28.01089.0</t>
+  </si>
+  <si>
+    <t>unang0110</t>
+  </si>
+  <si>
+    <t>pass pbb massal</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="7" x14ac:knownFonts="1">
+  <fonts count="9" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
@@ -657,6 +670,15 @@
       <name val="Calibri"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <charset val="1"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -849,50 +871,56 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="29">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="3" xfId="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="4" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="5" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="5" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="7" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="14" fontId="2" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="8" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="8" xfId="1" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="10" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="5" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="49" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="14" fontId="1" fillId="0" borderId="11" xfId="1" applyNumberFormat="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="11" xfId="1" quotePrefix="1" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="12" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="8" xfId="2" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
+    <cellStyle name="Hyperlink" xfId="2" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Normal 2" xfId="1" xr:uid="{8721F785-B009-4045-8755-1F86CCCA867C}"/>
   </cellStyles>
@@ -1200,7 +1228,7 @@
     <outlinePr summaryBelow="0" summaryRight="0"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:M22"/>
+  <dimension ref="A1:N22"/>
   <sheetFormatPr defaultColWidth="12.54296875" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="4.26953125" style="5" customWidth="1"/>
@@ -1220,7 +1248,7 @@
     <col min="19" max="16384" width="12.54296875" style="5"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:14" ht="30.75" customHeight="1" thickBot="1" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>1</v>
       </c>
@@ -1260,8 +1288,11 @@
       <c r="M1" s="4" t="s">
         <v>12</v>
       </c>
+      <c r="N1" s="5" t="s">
+        <v>188</v>
+      </c>
     </row>
-    <row r="2" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A2" s="6">
         <v>1</v>
       </c>
@@ -1302,7 +1333,7 @@
         <v>22</v>
       </c>
     </row>
-    <row r="3" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A3" s="13">
         <v>2</v>
       </c>
@@ -1315,7 +1346,7 @@
       <c r="D3" s="15" t="s">
         <v>24</v>
       </c>
-      <c r="E3" s="16" t="s">
+      <c r="E3" s="29" t="s">
         <v>25</v>
       </c>
       <c r="F3" s="15" t="s">
@@ -1324,10 +1355,10 @@
       <c r="G3" s="17">
         <v>27370</v>
       </c>
-      <c r="H3" s="15" t="s">
+      <c r="H3" s="30" t="s">
         <v>27</v>
       </c>
-      <c r="I3" s="18" t="s">
+      <c r="I3" s="31" t="s">
         <v>28</v>
       </c>
       <c r="J3" s="15" t="s">
@@ -1336,14 +1367,17 @@
       <c r="K3" s="15" t="s">
         <v>20</v>
       </c>
-      <c r="L3" s="15" t="s">
+      <c r="L3" s="32" t="s">
         <v>30</v>
       </c>
       <c r="M3" s="19" t="s">
         <v>31</v>
       </c>
+      <c r="N3" s="5" t="s">
+        <v>187</v>
+      </c>
     </row>
-    <row r="4" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A4" s="13">
         <v>3</v>
       </c>
@@ -1384,7 +1418,7 @@
         <v>40</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A5" s="13">
         <v>4</v>
       </c>
@@ -1425,7 +1459,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="6" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A6" s="13">
         <v>5</v>
       </c>
@@ -1466,7 +1500,7 @@
         <v>57</v>
       </c>
     </row>
-    <row r="7" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A7" s="13">
         <v>6</v>
       </c>
@@ -1507,7 +1541,7 @@
         <v>65</v>
       </c>
     </row>
-    <row r="8" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A8" s="13">
         <v>7</v>
       </c>
@@ -1548,7 +1582,7 @@
         <v>73</v>
       </c>
     </row>
-    <row r="9" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A9" s="13">
         <v>8</v>
       </c>
@@ -1589,7 +1623,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="10" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A10" s="13">
         <v>9</v>
       </c>
@@ -1630,7 +1664,7 @@
         <v>89</v>
       </c>
     </row>
-    <row r="11" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A11" s="13">
         <v>10</v>
       </c>
@@ -1671,7 +1705,7 @@
         <v>98</v>
       </c>
     </row>
-    <row r="12" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A12" s="13">
         <v>11</v>
       </c>
@@ -1712,7 +1746,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="13" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A13" s="13">
         <v>12</v>
       </c>
@@ -1753,7 +1787,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="14" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A14" s="13">
         <v>13</v>
       </c>
@@ -1794,7 +1828,7 @@
         <v>123</v>
       </c>
     </row>
-    <row r="15" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A15" s="13">
         <v>14</v>
       </c>
@@ -1835,7 +1869,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="16" spans="1:13" ht="14.5" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:14" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A16" s="13">
         <v>15</v>
       </c>
@@ -2123,7 +2157,10 @@
       </c>
     </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="L3" r:id="rId1" xr:uid="{E7C8ACF6-34FF-4635-8356-64D8C78650C5}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="5" fitToHeight="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId1"/>
+  <pageSetup paperSize="5" fitToHeight="0" orientation="portrait" horizontalDpi="4294967293" verticalDpi="0" r:id="rId2"/>
 </worksheet>
 </file>
</xml_diff>